<commit_message>
Handle ambiguous party benchmark cases in accuracy pipeline
Adds targeted exclusions and modal benchmark overrides for cases where the raw modal benchmark category is Other but is not comparable to the CES response structure.

Skips the 2014 Florida U.S. House District 23 candidate-level comparison because CES appears to have listed Debbie Wasserman Schultz with the wrong party label, and excludes the same district from the 2014 Florida House party-level CES and benchmark calculations for parity.

Forces selected candidate- and party-level benchmarks to major-party comparisons when independent or Other winners would otherwise drive the modal benchmark, including Rhode Island Governor 2010 and North Dakota Secretary of State 2018.

Keeps ambiguous Mississippi state legislative special/nonpartisan races excluded through the skip conditions table, where respondent interpretation and benchmark party labels cannot be validated consistently.
</commit_message>
<xml_diff>
--- a/data/Benchmarks/Election Returns/Governor_Returns_2006_2022.xlsx
+++ b/data/Benchmarks/Election Returns/Governor_Returns_2006_2022.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jdpruett/Desktop/CES Accuracy Analysis/data/Election Validation/Final Sets - Clean Fixed/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jdpruett/Desktop/CES Accuracy Analysis/data/Benchmarks/Election Returns/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C08393DD-A83E-2D4A-9C1F-15795EAAB283}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF387911-8322-8544-A9C2-F24C38831327}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2380" yWindow="1020" windowWidth="24220" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8780" uniqueCount="1020">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8783" uniqueCount="1020">
   <si>
     <t>year</t>
   </si>
@@ -46046,6 +46046,9 @@
       <c r="P829">
         <v>2</v>
       </c>
+      <c r="Q829" t="s">
+        <v>324</v>
+      </c>
     </row>
     <row r="830" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A830">
@@ -46097,6 +46100,9 @@
       <c r="P830">
         <v>1</v>
       </c>
+      <c r="Q830" t="s">
+        <v>324</v>
+      </c>
     </row>
     <row r="831" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A831">
@@ -46143,6 +46149,9 @@
       </c>
       <c r="O831" t="s">
         <v>31</v>
+      </c>
+      <c r="Q831" t="s">
+        <v>324</v>
       </c>
     </row>
     <row r="832" spans="1:17" x14ac:dyDescent="0.2">

</xml_diff>